<commit_message>
Ajout de meilleur commentaires, ordre méthode, import + simple
</commit_message>
<xml_diff>
--- a/validation.xlsx
+++ b/validation.xlsx
@@ -551,7 +551,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -600,6 +600,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF5EB91E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF8D1D75"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -709,7 +716,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -775,6 +782,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1942,7 +1953,7 @@
       <c r="A149" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B149" s="8"/>
+      <c r="B149" s="17"/>
     </row>
     <row r="150" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="7" t="s">
@@ -2128,7 +2139,7 @@
       <c r="A180" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B180" s="17"/>
+      <c r="B180" s="18"/>
     </row>
     <row r="181" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="5" t="s">
@@ -2140,13 +2151,13 @@
       <c r="A182" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B182" s="17"/>
+      <c r="B182" s="18"/>
     </row>
     <row r="183" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="B183" s="17"/>
+      <c r="B183" s="18"/>
     </row>
     <row r="184" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="5" t="s">
@@ -2158,13 +2169,13 @@
       <c r="A185" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="B185" s="17"/>
+      <c r="B185" s="18"/>
     </row>
     <row r="186" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="B186" s="17"/>
+      <c r="B186" s="18"/>
     </row>
     <row r="187" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="5" t="s">
@@ -2176,13 +2187,13 @@
       <c r="A188" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="B188" s="17"/>
+      <c r="B188" s="18"/>
     </row>
     <row r="189" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="B189" s="17"/>
+      <c r="B189" s="18"/>
     </row>
     <row r="190" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="5" t="s">
@@ -2194,19 +2205,19 @@
       <c r="A191" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="B191" s="17"/>
+      <c r="B191" s="18"/>
     </row>
     <row r="192" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="B192" s="17"/>
+      <c r="B192" s="18"/>
     </row>
     <row r="193" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B193" s="17"/>
+      <c r="B193" s="18"/>
     </row>
     <row r="194" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="5" t="s">
@@ -2218,37 +2229,37 @@
       <c r="A195" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="B195" s="17"/>
+      <c r="B195" s="18"/>
     </row>
     <row r="196" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="B196" s="17"/>
+      <c r="B196" s="18"/>
     </row>
     <row r="197" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="B197" s="17"/>
+      <c r="B197" s="18"/>
     </row>
     <row r="198" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="B198" s="17"/>
+      <c r="B198" s="18"/>
     </row>
     <row r="199" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="B199" s="17"/>
+      <c r="B199" s="18"/>
     </row>
     <row r="200" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="B200" s="17"/>
+      <c r="B200" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>